<commit_message>
Added the fields to the results sheet with URL statuscode and timestamp
</commit_message>
<xml_diff>
--- a/URLs.xlsx
+++ b/URLs.xlsx
@@ -1,26 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <x:workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/554380d165e11f13/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/554380d165e11f13/Documents/UiPath/CheckServerStatus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{124073A0-21C8-409F-B187-7DDCF6572F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C498A92F-DB5D-4477-804D-F3219C76ED7C}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{124073A0-21C8-409F-B187-7DDCF6572F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A92902AB-7394-45CE-9251-F119468BB766}"/>
+  <x:bookViews>
+    <x:workbookView xWindow="4335" yWindow="3885" windowWidth="17250" windowHeight="9015" firstSheet="0" activeTab="1" xr2:uid="{C498A92F-DB5D-4477-804D-F3219C76ED7C}"/>
+  </x:bookViews>
+  <x:sheets>
+    <x:sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <x:sheet name="Results" sheetId="2" r:id="rId2"/>
+  </x:sheets>
+  <x:definedNames/>
+  <x:calcPr calcId="191029"/>
+  <x:extLst>
+    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+    </x:ext>
+    <x:ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
@@ -30,87 +32,121 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+    </x:ext>
+  </x:extLst>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>https://amazon.com</t>
-  </si>
-  <si>
-    <t>https://www.google.com</t>
-  </si>
-  <si>
-    <t>https://www.thiswebsitedoesnotexist123.com</t>
-  </si>
-</sst>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:si>
+    <x:t>URL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.google.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://amazon.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.thiswebsitedoesnotexist123.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Status</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Timestamp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>text</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>ServiceUnavailable</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OK</x:t>
+  </x:si>
+</x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-  </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-  </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+<x:styleSheet xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac x16r2 xr">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="0" formatCode=""/>
+  </x:numFmts>
+  <x:fonts count="3" x14ac:knownFonts="1">
+    <x:font>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Aptos Narrow"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:u/>
+      <x:sz val="11"/>
+      <x:color theme="10"/>
+      <x:name val="Aptos Narrow"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="2">
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+  </x:fills>
+  <x:borders count="1">
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+  </x:borders>
+  <x:cellStyleXfs count="4">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="22" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+  </x:cellStyleXfs>
+  <x:cellXfs count="3">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <x:xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  </x:cellXfs>
+  <x:cellStyles count="2">
+    <x:cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </x:cellStyles>
+  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <x:extLst>
+    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+    </x:ext>
+    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
-</styleSheet>
+    </x:ext>
+  </x:extLst>
+</x:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -429,35 +465,163 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A2446D2-CE6A-4A64-B64A-147AA652A8AD}">
-  <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{AF653AB5-DE30-43C3-81F5-12A989BDA3F2}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{A4FAE71C-1E82-4B9E-8015-618E32EAA594}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xr:uid="{8A2446D2-CE6A-4A64-B64A-147AA652A8AD}" mc:Ignorable="x14ac xr xr2 xr3">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:A4"/>
+  <x:sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <x:sheetData>
+    <x:row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <x:c r="A1" s="0" t="s">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <x:c r="A2" s="1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <x:c r="A3" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <x:c r="A4" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:hyperlinks>
+    <x:hyperlink ref="A2" r:id="rId10"/>
+    <x:hyperlink ref="A3" r:id="rId11"/>
+  </x:hyperlinks>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xr:uid="{21B0C07D-CC04-43ED-8932-FB777046ABE9}" mc:Ignorable="x14ac xr xr2 xr3">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:C3"/>
+  <x:sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <x:cols>
+    <x:col min="1" max="1" width="41.855469" style="0" bestFit="1" customWidth="1"/>
+    <x:col min="2" max="2" width="18" style="0" bestFit="1" customWidth="1"/>
+    <x:col min="3" max="3" width="15.570312" style="0" bestFit="1" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A1" s="0" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A2" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <x:c r="A3" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C3" s="2">
+        <x:v>46126.9465046296</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:3">
+      <x:c r="A4" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:3">
+      <x:c r="A5" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C5" s="2">
+        <x:v>46126.9472685185</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:3">
+      <x:c r="A6" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:3">
+      <x:c r="A7" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C7" s="2">
+        <x:v>46126.9473032407</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:3">
+      <x:c r="A8" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:3">
+      <x:c r="A9" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C9" s="2">
+        <x:v>46126.9473148148</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Added try catch block to handle unreachable servers
</commit_message>
<xml_diff>
--- a/URLs.xlsx
+++ b/URLs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <x:workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+<x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <x:workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/554380d165e11f13/Documents/UiPath/CheckServerStatus/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3c1d036273c4525f/Documents/UiPath/server-health-checker-bot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{124073A0-21C8-409F-B187-7DDCF6572F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A92902AB-7394-45CE-9251-F119468BB766}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{124073A0-21C8-409F-B187-7DDCF6572F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31099E35-5D39-4782-914C-044B861C8338}"/>
   <x:bookViews>
-    <x:workbookView xWindow="4335" yWindow="3885" windowWidth="17250" windowHeight="9015" firstSheet="0" activeTab="1" xr2:uid="{C498A92F-DB5D-4477-804D-F3219C76ED7C}"/>
+    <x:workbookView xWindow="2205" yWindow="2205" windowWidth="15375" windowHeight="7785" firstSheet="0" activeTab="0" xr2:uid="{C498A92F-DB5D-4477-804D-F3219C76ED7C}"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,9 +29,10 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </x:ext>
+    <x:ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </x:ext>
   </x:extLst>
 </x:workbook>
@@ -52,22 +53,19 @@
     <x:t>https://www.thiswebsitedoesnotexist123.com</x:t>
   </x:si>
   <x:si>
+    <x:t>https://www.fakeserver99999.com</x:t>
+  </x:si>
+  <x:si>
     <x:t>Status</x:t>
   </x:si>
   <x:si>
     <x:t>Timestamp</x:t>
   </x:si>
   <x:si>
-    <x:t>text</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
+    <x:t>OK</x:t>
   </x:si>
   <x:si>
     <x:t>ServiceUnavailable</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OK</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -77,7 +75,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="0" formatCode=""/>
   </x:numFmts>
-  <x:fonts count="3" x14ac:knownFonts="1">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -469,33 +467,38 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:A4"/>
-  <x:sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <x:dimension ref="A1:A5"/>
+  <x:sheetFormatPr defaultRowHeight="14.25"/>
   <x:sheetData>
-    <x:row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <x:row r="1" spans="1:1">
       <x:c r="A1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <x:row r="2" spans="1:1">
       <x:c r="A2" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <x:row r="3" spans="1:1">
       <x:c r="A3" s="1" t="s">
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <x:row r="4" spans="1:1">
       <x:c r="A4" s="0" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
+    <x:row r="5" spans="1:1">
+      <x:c r="A5" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink ref="A2" r:id="rId10"/>
-    <x:hyperlink ref="A3" r:id="rId11"/>
+    <x:hyperlink ref="A2" r:id="rId8"/>
+    <x:hyperlink ref="A3" r:id="rId9"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -510,56 +513,56 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C3"/>
-  <x:sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <x:dimension ref="A1:C9"/>
+  <x:sheetFormatPr defaultRowHeight="14.25"/>
   <x:cols>
-    <x:col min="1" max="1" width="41.855469" style="0" bestFit="1" customWidth="1"/>
+    <x:col min="1" max="1" width="41.875" style="0" bestFit="1" customWidth="1"/>
     <x:col min="2" max="2" width="18" style="0" bestFit="1" customWidth="1"/>
-    <x:col min="3" max="3" width="15.570312" style="0" bestFit="1" customWidth="1"/>
+    <x:col min="3" max="3" width="15.625" style="0" bestFit="1" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <x:row r="1" spans="1:3">
       <x:c r="A1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C2" s="0" t="s">
+      <x:c r="C2" s="2">
+        <x:v>46127.7355324074</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:3">
+      <x:c r="A3" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <x:c r="A3" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
       <x:c r="C3" s="2">
-        <x:v>46126.9465046296</x:v>
+        <x:v>46127.7359722222</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C4" s="2">
+        <x:v>46127.7361458333</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3">
@@ -567,54 +570,87 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C5" s="2">
-        <x:v>46126.9472685185</x:v>
+        <x:v>46127.8119907407</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>7</x:v>
+      <x:c r="C6" s="2">
+        <x:v>46127.8120949074</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="0" t="s">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C7" s="2">
-        <x:v>46126.9473032407</x:v>
+        <x:v>46127.8121180556</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:3">
       <x:c r="A8" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C8" s="2">
+        <x:v>46127.8121296296</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:3">
       <x:c r="A9" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C9" s="2">
+        <x:v>46127.814224537</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:3">
+      <x:c r="A10" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C10" s="2">
+        <x:v>46127.8142708333</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:3">
+      <x:c r="A11" s="0" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B9" s="0" t="s">
+      <x:c r="B11" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="C9" s="2">
-        <x:v>46126.9473148148</x:v>
+      <x:c r="C11" s="2">
+        <x:v>46127.8142939815</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:3">
+      <x:c r="A12" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C12" s="2">
+        <x:v>46127.8143055556</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>